<commit_message>
Point image list links at the Vercel site
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Ouroboros - Website Image List.xlsx
+++ b/Ouroboros - Website Image List.xlsx
@@ -43,7 +43,7 @@
     <t>Front view of the lodge on a clear, sunny day with the mountains and river behind. Same camera spot as hero-snow.jpg.</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/infindigital/ouroboros/main/assets/img/new/hero-autumn.jpg</t>
+    <t>https://infindigital-ouroboros.vercel.app/assets/img/new/hero-autumn.jpg</t>
   </si>
   <si>
     <t>hero-snow.jpg</t>
@@ -52,7 +52,7 @@
     <t>The same front view of the lodge covered in snow. Same camera spot as hero-autumn.jpg.</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/infindigital/ouroboros/main/assets/img/new/hero-snow.jpg</t>
+    <t>https://infindigital-ouroboros.vercel.app/assets/img/new/hero-snow.jpg</t>
   </si>
   <si>
     <t>exterior-autumn.jpg</t>
@@ -64,7 +64,7 @@
     <t>Outside of the property in autumn or summer, with the village and mountains around it. Same camera spot as exterior-snow.jpg.</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/infindigital/ouroboros/main/assets/img/exterior-autumn.jpg</t>
+    <t>https://infindigital-ouroboros.vercel.app/assets/img/exterior-autumn.jpg</t>
   </si>
   <si>
     <t>exterior-snow.jpg</t>
@@ -73,7 +73,7 @@
     <t>The same outside view of the property in winter snow. Same camera spot as exterior-autumn.jpg.</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/infindigital/ouroboros/main/assets/img/exterior-snow.jpg</t>
+    <t>https://infindigital-ouroboros.vercel.app/assets/img/exterior-snow.jpg</t>
   </si>
   <si>
     <t>suite-view.jpg</t>
@@ -82,7 +82,7 @@
     <t>The Mountain Suite: the red bed with the balcony doors and the mountain view.</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/infindigital/ouroboros/main/assets/img/new/suite-view.jpg</t>
+    <t>https://infindigital-ouroboros.vercel.app/assets/img/new/suite-view.jpg</t>
   </si>
   <si>
     <t>room-balcony.jpg</t>
@@ -91,7 +91,7 @@
     <t>The Balcony Room: bed and the floor-to-ceiling windows facing the mountains.</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/infindigital/ouroboros/main/assets/img/room-balcony.jpg</t>
+    <t>https://infindigital-ouroboros.vercel.app/assets/img/room-balcony.jpg</t>
   </si>
   <si>
     <t>room-crimson.jpg</t>
@@ -100,7 +100,7 @@
     <t>The Crimson Room: red headboard, armchairs and sitting nook.</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/infindigital/ouroboros/main/assets/img/room-crimson.jpg</t>
+    <t>https://infindigital-ouroboros.vercel.app/assets/img/room-crimson.jpg</t>
   </si>
   <si>
     <t>room-crimson-top.jpg</t>
@@ -112,7 +112,7 @@
     <t>The Crimson Room photographed from above or a high corner, showing the bed and linen.</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/infindigital/ouroboros/main/assets/img/room-crimson-top.jpg</t>
+    <t>https://infindigital-ouroboros.vercel.app/assets/img/room-crimson-top.jpg</t>
   </si>
   <si>
     <t>room-suite.jpg</t>
@@ -121,7 +121,7 @@
     <t>The Sanctuary room: large bed, sheer curtains and soft daylight.</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/infindigital/ouroboros/main/assets/img/room-suite.jpg</t>
+    <t>https://infindigital-ouroboros.vercel.app/assets/img/room-suite.jpg</t>
   </si>
   <si>
     <t>bathtub.jpg</t>
@@ -130,7 +130,7 @@
     <t>The bathtub next to the big window with the river and mountain view.</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/infindigital/ouroboros/main/assets/img/bathtub.jpg</t>
+    <t>https://infindigital-ouroboros.vercel.app/assets/img/bathtub.jpg</t>
   </si>
   <si>
     <t>spa-bath.jpg</t>
@@ -139,7 +139,7 @@
     <t>A bathroom with the tub and a mountain view, from a different angle than bathtub.jpg.</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/infindigital/ouroboros/main/assets/img/new/spa-bath.jpg</t>
+    <t>https://infindigital-ouroboros.vercel.app/assets/img/new/spa-bath.jpg</t>
   </si>
   <si>
     <t>rose-bath.jpg</t>
@@ -151,7 +151,7 @@
     <t>The scenic bathtub facing the mountains, close-up.</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/infindigital/ouroboros/main/assets/img/new/rose-bath.jpg</t>
+    <t>https://infindigital-ouroboros.vercel.app/assets/img/new/rose-bath.jpg</t>
   </si>
   <si>
     <t>firepit-sunset.jpg</t>
@@ -160,7 +160,7 @@
     <t>The terrace bonfire lit at sunset.</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/infindigital/ouroboros/main/assets/img/new/firepit-sunset.jpg</t>
+    <t>https://infindigital-ouroboros.vercel.app/assets/img/new/firepit-sunset.jpg</t>
   </si>
   <si>
     <t>snow-firelight.jpg</t>
@@ -169,7 +169,7 @@
     <t>The terrace in snow with the bonfire glowing.</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/infindigital/ouroboros/main/assets/img/new/snow-firelight.jpg</t>
+    <t>https://infindigital-ouroboros.vercel.app/assets/img/new/snow-firelight.jpg</t>
   </si>
   <si>
     <t>breakfast-terrace.jpg</t>
@@ -178,7 +178,7 @@
     <t>Breakfast served with the valley view.</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/infindigital/ouroboros/main/assets/img/new/breakfast-terrace.jpg</t>
+    <t>https://infindigital-ouroboros.vercel.app/assets/img/new/breakfast-terrace.jpg</t>
   </si>
   <si>
     <t>terrace-lounge.jpg</t>
@@ -187,7 +187,7 @@
     <t>Terrace or seating area at golden hour with the mountains behind.</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/infindigital/ouroboros/main/assets/img/new/terrace-lounge.jpg</t>
+    <t>https://infindigital-ouroboros.vercel.app/assets/img/new/terrace-lounge.jpg</t>
   </si>
   <si>
     <t>terrace-river.jpg</t>
@@ -196,7 +196,7 @@
     <t>Terrace or seating area looking out over the river valley.</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/infindigital/ouroboros/main/assets/img/new/terrace-river.jpg</t>
+    <t>https://infindigital-ouroboros.vercel.app/assets/img/new/terrace-river.jpg</t>
   </si>
   <si>
     <t>himachali-food.jpg</t>
@@ -205,7 +205,7 @@
     <t>A home-cooked Himachali meal served at the property.</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/infindigital/ouroboros/main/assets/img/stock/himachali-food.jpg</t>
+    <t>https://infindigital-ouroboros.vercel.app/assets/img/stock/himachali-food.jpg</t>
   </si>
   <si>
     <t>chandra-valley.jpg</t>
@@ -214,7 +214,7 @@
     <t>The Chandra River winding through the valley near Koksar.</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/infindigital/ouroboros/main/assets/img/chandra-valley.jpg</t>
+    <t>https://infindigital-ouroboros.vercel.app/assets/img/chandra-valley.jpg</t>
   </si>
   <si>
     <t>peaks-dusk.jpg</t>
@@ -223,7 +223,7 @@
     <t>Snow peaks around Lahaul glowing at dusk.</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/infindigital/ouroboros/main/assets/img/peaks-dusk.jpg</t>
+    <t>https://infindigital-ouroboros.vercel.app/assets/img/peaks-dusk.jpg</t>
   </si>
   <si>
     <t>mountain-pines.jpg</t>
@@ -232,7 +232,7 @@
     <t>The Atal Tunnel or the mountain road leading to Koksar.</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/infindigital/ouroboros/main/assets/img/stock/mountain-pines.jpg</t>
+    <t>https://infindigital-ouroboros.vercel.app/assets/img/stock/mountain-pines.jpg</t>
   </si>
   <si>
     <t>lake.jpg</t>
@@ -241,7 +241,7 @@
     <t>Sissu Lake.</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/infindigital/ouroboros/main/assets/img/stock/lake.jpg</t>
+    <t>https://infindigital-ouroboros.vercel.app/assets/img/stock/lake.jpg</t>
   </si>
   <si>
     <t>waterfall.jpg</t>
@@ -250,7 +250,7 @@
     <t>Sissu Waterfall.</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/infindigital/ouroboros/main/assets/img/stock/waterfall.jpg</t>
+    <t>https://infindigital-ouroboros.vercel.app/assets/img/stock/waterfall.jpg</t>
   </si>
   <si>
     <t>monastery.jpg</t>
@@ -259,7 +259,7 @@
     <t>A monastery in Keylong or nearby.</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/infindigital/ouroboros/main/assets/img/stock/monastery.jpg</t>
+    <t>https://infindigital-ouroboros.vercel.app/assets/img/stock/monastery.jpg</t>
   </si>
   <si>
     <t>snow-play.jpg</t>
@@ -268,7 +268,7 @@
     <t>Guests playing in the snow or building a snowman near the property.</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/infindigital/ouroboros/main/assets/img/stock/snow-play.jpg</t>
+    <t>https://infindigital-ouroboros.vercel.app/assets/img/stock/snow-play.jpg</t>
   </si>
   <si>
     <t>sunrise.jpg</t>
@@ -277,7 +277,7 @@
     <t>Sunrise or sunset over the mountains, ideally taken from the property.</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/infindigital/ouroboros/main/assets/img/stock/sunrise.jpg</t>
+    <t>https://infindigital-ouroboros.vercel.app/assets/img/stock/sunrise.jpg</t>
   </si>
   <si>
     <t>village-walk.jpg</t>
@@ -286,7 +286,7 @@
     <t>A walk on a village trail around Koksar.</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/infindigital/ouroboros/main/assets/img/stock/village-walk.jpg</t>
+    <t>https://infindigital-ouroboros.vercel.app/assets/img/stock/village-walk.jpg</t>
   </si>
   <si>
     <t>logo-horizontal.png</t>
@@ -298,7 +298,7 @@
     <t>Main logo (emblem + OUROBOROS HOSPITALITY) in colour, transparent background. PNG or SVG.</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/infindigital/ouroboros/main/assets/img/logo-horizontal.png</t>
+    <t>https://infindigital-ouroboros.vercel.app/assets/img/logo-horizontal.png</t>
   </si>
   <si>
     <t>logo-horizontal-light.png</t>
@@ -307,7 +307,7 @@
     <t>The same logo in white and gold for dark backgrounds, transparent background. PNG or SVG.</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/infindigital/ouroboros/main/assets/img/logo-horizontal-light.png</t>
+    <t>https://infindigital-ouroboros.vercel.app/assets/img/logo-horizontal-light.png</t>
   </si>
   <si>
     <t>logo-emblem.png</t>
@@ -319,7 +319,7 @@
     <t>The Q emblem on its own (no text), transparent background. PNG or SVG.</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/infindigital/ouroboros/main/assets/img/logo-emblem.png</t>
+    <t>https://infindigital-ouroboros.vercel.app/assets/img/logo-emblem.png</t>
   </si>
   <si>
     <t>favicon.png</t>
@@ -331,7 +331,7 @@
     <t>The Q emblem as a small square icon for the browser tab.</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/infindigital/ouroboros/main/assets/img/favicon.png</t>
+    <t>https://infindigital-ouroboros.vercel.app/assets/img/favicon.png</t>
   </si>
   <si>
     <t>apple-touch-icon.png</t>
@@ -343,7 +343,7 @@
     <t>The Q emblem as a square icon for phone home screens.</t>
   </si>
   <si>
-    <t>https://raw.githubusercontent.com/infindigital/ouroboros/main/assets/img/apple-touch-icon.png</t>
+    <t>https://infindigital-ouroboros.vercel.app/assets/img/apple-touch-icon.png</t>
   </si>
 </sst>
 </file>

</xml_diff>